<commit_message>
converted to sqlite database
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -521,7 +521,11 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -554,7 +558,11 @@
           <t>10:30</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>